<commit_message>
includes data used for imputation
</commit_message>
<xml_diff>
--- a/data/data-matrix.xlsx
+++ b/data/data-matrix.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eggert\Desktop\d-20231020-I30-Anne-MarieGalow_Schweine\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\FBNGroup\I2-StatConsult\d-data-analysis\d-20231020-I30-Anne-MarieGalow_Schweine\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AEFC5DC-986A-4D40-92CF-EEB5679D4172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12AF2EB-EF2A-45C5-82F6-1ADE3ABFC1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_ori" sheetId="2" r:id="rId1"/>
-    <sheet name="data_imp" sheetId="5" r:id="rId2"/>
-    <sheet name="parameter_description" sheetId="3" r:id="rId3"/>
+    <sheet name="data_ori_knn" sheetId="6" r:id="rId2"/>
+    <sheet name="data_imp" sheetId="5" r:id="rId3"/>
+    <sheet name="parameter_description" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="65">
   <si>
     <t>housing</t>
   </si>
@@ -4410,6 +4411,1999 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{276C3199-2A25-4CB5-85A0-610600A578D9}">
+  <dimension ref="A1:R43"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="14.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" style="4" bestFit="1"/>
+    <col min="5" max="5" width="12.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5703125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="16384" width="14.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="4">
+        <v>6733</v>
+      </c>
+      <c r="C2" s="4">
+        <v>226</v>
+      </c>
+      <c r="D2" s="5">
+        <v>15.692457554098473</v>
+      </c>
+      <c r="E2" s="5">
+        <v>8.142018712873341</v>
+      </c>
+      <c r="F2" s="5">
+        <v>394.11095866489234</v>
+      </c>
+      <c r="G2" s="5">
+        <v>406.75366409057744</v>
+      </c>
+      <c r="H2" s="5">
+        <v>595.49751987073842</v>
+      </c>
+      <c r="I2" s="5">
+        <v>54.141399999999997</v>
+      </c>
+      <c r="J2" s="5">
+        <v>90.545029999999997</v>
+      </c>
+      <c r="K2" s="5">
+        <v>54.380600000000001</v>
+      </c>
+      <c r="L2" s="5">
+        <v>198.81490500000001</v>
+      </c>
+      <c r="M2" s="6">
+        <v>698.72289000000001</v>
+      </c>
+      <c r="N2" s="6">
+        <v>510.60470000000004</v>
+      </c>
+      <c r="O2" s="6">
+        <v>994.150665</v>
+      </c>
+      <c r="P2" s="6">
+        <v>4922.4711950000001</v>
+      </c>
+      <c r="Q2" s="6">
+        <v>161.25561356544495</v>
+      </c>
+      <c r="R2" s="6">
+        <v>95.634143710136414</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="4">
+        <v>6733</v>
+      </c>
+      <c r="C3" s="4">
+        <v>247</v>
+      </c>
+      <c r="D3" s="5">
+        <v>8.2192665752898098</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.87179495566672072</v>
+      </c>
+      <c r="F3" s="5">
+        <v>273.96052666541277</v>
+      </c>
+      <c r="G3" s="5">
+        <v>330.08187636282383</v>
+      </c>
+      <c r="H3" s="5">
+        <v>394.78387860224825</v>
+      </c>
+      <c r="I3" s="5">
+        <v>47.8645</v>
+      </c>
+      <c r="J3" s="5">
+        <v>85.026949999999999</v>
+      </c>
+      <c r="K3" s="5">
+        <v>215.46451999999999</v>
+      </c>
+      <c r="L3" s="5">
+        <v>291.33449999999999</v>
+      </c>
+      <c r="M3" s="6">
+        <v>497.07729999999998</v>
+      </c>
+      <c r="N3" s="6">
+        <v>403.47739999999999</v>
+      </c>
+      <c r="O3" s="6">
+        <v>386.48615000000001</v>
+      </c>
+      <c r="P3" s="6">
+        <v>309.9042</v>
+      </c>
+      <c r="Q3" s="6">
+        <v>2429.7113262414932</v>
+      </c>
+      <c r="R3" s="6">
+        <v>1282.9630436897278</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="4">
+        <v>6733</v>
+      </c>
+      <c r="C4" s="4">
+        <v>316</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5">
+        <v>126.24208272197774</v>
+      </c>
+      <c r="G4" s="5">
+        <v>222.19936914337904</v>
+      </c>
+      <c r="H4" s="5">
+        <v>201.60826116464125</v>
+      </c>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="6">
+        <v>674.911206666667</v>
+      </c>
+      <c r="N4" s="6">
+        <v>494.125766666667</v>
+      </c>
+      <c r="O4" s="6">
+        <v>1627.2419725</v>
+      </c>
+      <c r="P4" s="6">
+        <v>1530.2762299999999</v>
+      </c>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="4">
+        <v>6734</v>
+      </c>
+      <c r="C5" s="4">
+        <v>226</v>
+      </c>
+      <c r="D5" s="5">
+        <v>25.955737364195709</v>
+      </c>
+      <c r="E5" s="5">
+        <v>3.7280194082784939</v>
+      </c>
+      <c r="F5" s="5">
+        <v>437.31834668909181</v>
+      </c>
+      <c r="G5" s="5">
+        <v>400.24589892574994</v>
+      </c>
+      <c r="H5" s="5">
+        <v>305.42453804250295</v>
+      </c>
+      <c r="I5" s="5">
+        <v>114.68749</v>
+      </c>
+      <c r="J5" s="5">
+        <v>122.19062</v>
+      </c>
+      <c r="K5" s="5">
+        <v>322.41636</v>
+      </c>
+      <c r="L5" s="5">
+        <v>336.48054999999999</v>
+      </c>
+      <c r="M5" s="6">
+        <v>487.92964999999998</v>
+      </c>
+      <c r="N5" s="6">
+        <v>498.14749999999998</v>
+      </c>
+      <c r="O5" s="6">
+        <v>419.66404999999997</v>
+      </c>
+      <c r="P5" s="6">
+        <v>354.95184999999998</v>
+      </c>
+      <c r="Q5" s="6">
+        <v>4672.3250069618225</v>
+      </c>
+      <c r="R5" s="6">
+        <v>2255.1267460584641</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="4">
+        <v>6734</v>
+      </c>
+      <c r="C6" s="4">
+        <v>247</v>
+      </c>
+      <c r="D6" s="5">
+        <v>6.7337036228278189</v>
+      </c>
+      <c r="E6" s="5">
+        <v>5.2275392750001517</v>
+      </c>
+      <c r="F6" s="5">
+        <v>521.88466580574902</v>
+      </c>
+      <c r="G6" s="5">
+        <v>548.91586616663994</v>
+      </c>
+      <c r="H6" s="5">
+        <v>484.52099167868573</v>
+      </c>
+      <c r="I6" s="5">
+        <v>51.447839999999999</v>
+      </c>
+      <c r="J6" s="5">
+        <v>105.3578</v>
+      </c>
+      <c r="K6" s="5">
+        <v>362.08983999999998</v>
+      </c>
+      <c r="L6" s="5">
+        <v>222.5128</v>
+      </c>
+      <c r="M6" s="6">
+        <v>858.14679999999998</v>
+      </c>
+      <c r="N6" s="6">
+        <v>795.68079999999998</v>
+      </c>
+      <c r="O6" s="6">
+        <v>633.77705000000003</v>
+      </c>
+      <c r="P6" s="6">
+        <v>356.59010000000001</v>
+      </c>
+      <c r="Q6" s="6">
+        <v>8402.5168563127518</v>
+      </c>
+      <c r="R6" s="6">
+        <v>8630.4036334753036</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="4">
+        <v>6734</v>
+      </c>
+      <c r="C7" s="4">
+        <v>316</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5">
+        <v>42.506588673482042</v>
+      </c>
+      <c r="G7" s="5">
+        <v>55.419458299707813</v>
+      </c>
+      <c r="H7" s="5">
+        <v>26.482359964693643</v>
+      </c>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="6">
+        <v>373.97332</v>
+      </c>
+      <c r="N7" s="6">
+        <v>524.44722000000002</v>
+      </c>
+      <c r="O7" s="6">
+        <v>1874.4859199999999</v>
+      </c>
+      <c r="P7" s="6">
+        <v>4932.4301699999996</v>
+      </c>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="4">
+        <v>6791</v>
+      </c>
+      <c r="C8" s="4">
+        <v>247</v>
+      </c>
+      <c r="D8" s="5">
+        <v>10.584995891062277</v>
+      </c>
+      <c r="E8" s="5">
+        <v>4.7676710713933712</v>
+      </c>
+      <c r="F8" s="5">
+        <v>385.13804427840881</v>
+      </c>
+      <c r="G8" s="5">
+        <v>342.22296861075762</v>
+      </c>
+      <c r="H8" s="5">
+        <v>218.51018010576897</v>
+      </c>
+      <c r="I8" s="5">
+        <v>59.54401</v>
+      </c>
+      <c r="J8" s="5">
+        <v>99.786389999999997</v>
+      </c>
+      <c r="K8" s="5">
+        <v>50.639000000000003</v>
+      </c>
+      <c r="L8" s="5">
+        <v>90.572000000000003</v>
+      </c>
+      <c r="M8" s="6">
+        <v>665.29670999999996</v>
+      </c>
+      <c r="N8" s="6">
+        <v>477.07975999999996</v>
+      </c>
+      <c r="O8" s="6">
+        <v>780.46623999999997</v>
+      </c>
+      <c r="P8" s="6">
+        <v>1430.3273750000001</v>
+      </c>
+      <c r="Q8" s="6">
+        <v>78.41329300403595</v>
+      </c>
+      <c r="R8" s="6">
+        <v>49.892759799957275</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="4">
+        <v>6791</v>
+      </c>
+      <c r="C9" s="4">
+        <v>316</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5">
+        <v>143.48436932687633</v>
+      </c>
+      <c r="G9" s="5">
+        <v>180.13372088516746</v>
+      </c>
+      <c r="H9" s="5">
+        <v>147.85493244269833</v>
+      </c>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="6">
+        <v>538.76927250000006</v>
+      </c>
+      <c r="N9" s="6">
+        <v>946.69412750000004</v>
+      </c>
+      <c r="O9" s="6">
+        <v>758.34581249999997</v>
+      </c>
+      <c r="P9" s="6">
+        <v>1738.6462025000001</v>
+      </c>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="4">
+        <v>6791</v>
+      </c>
+      <c r="C10" s="4">
+        <v>337</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5">
+        <v>97.526395927838536</v>
+      </c>
+      <c r="G10" s="5">
+        <v>121.45027169048856</v>
+      </c>
+      <c r="H10" s="5">
+        <v>85.891697603622845</v>
+      </c>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="4">
+        <v>6794</v>
+      </c>
+      <c r="C11" s="4">
+        <v>247</v>
+      </c>
+      <c r="D11" s="5">
+        <v>16.983810876059771</v>
+      </c>
+      <c r="E11" s="5">
+        <v>1.6193855415651486</v>
+      </c>
+      <c r="F11" s="5">
+        <v>411.68264744894554</v>
+      </c>
+      <c r="G11" s="5">
+        <v>531.09756983014415</v>
+      </c>
+      <c r="H11" s="5">
+        <v>492.55853163446227</v>
+      </c>
+      <c r="I11" s="5">
+        <v>62.253039999999999</v>
+      </c>
+      <c r="J11" s="5">
+        <v>110.94902999999999</v>
+      </c>
+      <c r="K11" s="5">
+        <v>47.600200000000001</v>
+      </c>
+      <c r="L11" s="5">
+        <v>185.76421999999999</v>
+      </c>
+      <c r="M11" s="6">
+        <v>606.95958000000007</v>
+      </c>
+      <c r="N11" s="6">
+        <v>461.37434000000002</v>
+      </c>
+      <c r="O11" s="6">
+        <v>603.12449000000004</v>
+      </c>
+      <c r="P11" s="6">
+        <v>1552.0043599999999</v>
+      </c>
+      <c r="Q11" s="6">
+        <v>37.399958252906799</v>
+      </c>
+      <c r="R11" s="6">
+        <v>35.318448662757874</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="4">
+        <v>6794</v>
+      </c>
+      <c r="C12" s="4">
+        <v>316</v>
+      </c>
+      <c r="D12" s="5">
+        <v>19.424758556832316</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2.8905360224016365</v>
+      </c>
+      <c r="F12" s="5">
+        <v>151.42636915112695</v>
+      </c>
+      <c r="G12" s="5">
+        <v>193.26045761821075</v>
+      </c>
+      <c r="H12" s="5">
+        <v>252.93738260080048</v>
+      </c>
+      <c r="I12" s="5">
+        <v>97.933679999999995</v>
+      </c>
+      <c r="J12" s="5">
+        <v>111.88283</v>
+      </c>
+      <c r="K12" s="5">
+        <v>263.21246000000002</v>
+      </c>
+      <c r="L12" s="5">
+        <v>404.15735999999998</v>
+      </c>
+      <c r="M12" s="6">
+        <v>678.28179999999998</v>
+      </c>
+      <c r="N12" s="6">
+        <v>583.42439999999999</v>
+      </c>
+      <c r="O12" s="6">
+        <v>260.38420000000002</v>
+      </c>
+      <c r="P12" s="6">
+        <v>304.79298</v>
+      </c>
+      <c r="Q12" s="6">
+        <v>3711.3905705213547</v>
+      </c>
+      <c r="R12" s="6">
+        <v>2518.1594341993332</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="4">
+        <v>6794</v>
+      </c>
+      <c r="C13" s="4">
+        <v>406</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5">
+        <v>49.756523773377914</v>
+      </c>
+      <c r="H13" s="5">
+        <v>56.512442471712191</v>
+      </c>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="6">
+        <v>658.71271249999995</v>
+      </c>
+      <c r="N13" s="6">
+        <v>705.42633750000005</v>
+      </c>
+      <c r="O13" s="6">
+        <v>1406.2753825</v>
+      </c>
+      <c r="P13" s="6">
+        <v>1055.9147049999999</v>
+      </c>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="4">
+        <v>6843</v>
+      </c>
+      <c r="C14" s="4">
+        <v>304</v>
+      </c>
+      <c r="D14" s="5">
+        <v>1.3308596642586965</v>
+      </c>
+      <c r="E14" s="5">
+        <v>2.7362891198099741</v>
+      </c>
+      <c r="F14" s="5">
+        <v>142.62882129585722</v>
+      </c>
+      <c r="G14" s="5">
+        <v>259.48294588656177</v>
+      </c>
+      <c r="H14" s="5">
+        <v>108.69333457044507</v>
+      </c>
+      <c r="I14" s="5">
+        <v>82.275469999999999</v>
+      </c>
+      <c r="J14" s="5">
+        <v>113.75206</v>
+      </c>
+      <c r="K14" s="5">
+        <v>93.957999999999998</v>
+      </c>
+      <c r="L14" s="5">
+        <v>127.098</v>
+      </c>
+      <c r="M14" s="6">
+        <v>1023.2126950000001</v>
+      </c>
+      <c r="N14" s="6">
+        <v>749.14460499999996</v>
+      </c>
+      <c r="O14" s="6">
+        <v>1753.225205</v>
+      </c>
+      <c r="P14" s="6">
+        <v>3545.1813999999999</v>
+      </c>
+      <c r="Q14" s="6">
+        <v>83.762903690338135</v>
+      </c>
+      <c r="R14" s="6">
+        <v>102.54687762260437</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="4">
+        <v>6843</v>
+      </c>
+      <c r="C15" s="4">
+        <v>325</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5">
+        <v>149.36194496341645</v>
+      </c>
+      <c r="G15" s="5">
+        <v>160.59176758173706</v>
+      </c>
+      <c r="H15" s="5">
+        <v>175.94396524024017</v>
+      </c>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="6">
+        <v>537.34787500000004</v>
+      </c>
+      <c r="N15" s="6">
+        <v>603.13457500000004</v>
+      </c>
+      <c r="O15" s="6">
+        <v>396.99618249999997</v>
+      </c>
+      <c r="P15" s="6">
+        <v>1896.1582375</v>
+      </c>
+      <c r="Q15" s="5"/>
+      <c r="R15" s="5"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="4">
+        <v>6843</v>
+      </c>
+      <c r="C16" s="4">
+        <v>346</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5">
+        <v>58.90084727366775</v>
+      </c>
+      <c r="G16" s="5">
+        <v>74.666379791878995</v>
+      </c>
+      <c r="H16" s="5">
+        <v>136.14169829884239</v>
+      </c>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="6">
+        <v>671.62824000000001</v>
+      </c>
+      <c r="N16" s="6">
+        <v>657.68354999999997</v>
+      </c>
+      <c r="O16" s="6">
+        <v>554.85607000000005</v>
+      </c>
+      <c r="P16" s="6">
+        <v>1595.1708699999999</v>
+      </c>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="4">
+        <v>6845</v>
+      </c>
+      <c r="C17" s="4">
+        <v>304</v>
+      </c>
+      <c r="D17" s="5">
+        <v>0.9594955024694245</v>
+      </c>
+      <c r="E17" s="5">
+        <v>12.59883996280025</v>
+      </c>
+      <c r="F17" s="5">
+        <v>106.6498524513687</v>
+      </c>
+      <c r="G17" s="5">
+        <v>64.200742980529512</v>
+      </c>
+      <c r="H17" s="5">
+        <v>68.697172823630723</v>
+      </c>
+      <c r="I17" s="5">
+        <v>86.864080000000001</v>
+      </c>
+      <c r="J17" s="5">
+        <v>154.46413999999999</v>
+      </c>
+      <c r="K17" s="5">
+        <v>74.102720000000005</v>
+      </c>
+      <c r="L17" s="5">
+        <v>222.79703000000001</v>
+      </c>
+      <c r="M17" s="6">
+        <v>1012.4522200000001</v>
+      </c>
+      <c r="N17" s="6">
+        <v>582.20501999999999</v>
+      </c>
+      <c r="O17" s="6">
+        <v>2454.6375800000001</v>
+      </c>
+      <c r="P17" s="6">
+        <v>3690.6158400000004</v>
+      </c>
+      <c r="Q17" s="6">
+        <v>41.210620164871216</v>
+      </c>
+      <c r="R17" s="6">
+        <v>40.491995096206665</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B18" s="4">
+        <v>6845</v>
+      </c>
+      <c r="C18" s="4">
+        <v>337</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5">
+        <v>194.95029547508992</v>
+      </c>
+      <c r="G18" s="5">
+        <v>133.44646953406868</v>
+      </c>
+      <c r="H18" s="5">
+        <v>120.99425490072247</v>
+      </c>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="6"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="6"/>
+      <c r="Q18" s="5"/>
+      <c r="R18" s="5"/>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B19" s="4">
+        <v>6924</v>
+      </c>
+      <c r="C19" s="4">
+        <v>325</v>
+      </c>
+      <c r="D19" s="5">
+        <v>58.138940874255773</v>
+      </c>
+      <c r="E19" s="5">
+        <v>3.8986067033384537</v>
+      </c>
+      <c r="F19" s="5">
+        <v>75.802342224046356</v>
+      </c>
+      <c r="G19" s="5">
+        <v>89.396683131617095</v>
+      </c>
+      <c r="H19" s="5">
+        <v>108.73236497660393</v>
+      </c>
+      <c r="I19" s="5">
+        <v>86.864080000000001</v>
+      </c>
+      <c r="J19" s="5">
+        <v>117.49708</v>
+      </c>
+      <c r="K19" s="5">
+        <v>296.75312000000002</v>
+      </c>
+      <c r="L19" s="5">
+        <v>341.4085</v>
+      </c>
+      <c r="M19" s="6">
+        <v>615.37779999999998</v>
+      </c>
+      <c r="N19" s="6">
+        <v>898.90634999999997</v>
+      </c>
+      <c r="O19" s="6">
+        <v>455.01330000000002</v>
+      </c>
+      <c r="P19" s="6">
+        <v>650.48650999999995</v>
+      </c>
+      <c r="Q19" s="6">
+        <v>142.26887357234955</v>
+      </c>
+      <c r="R19" s="6">
+        <v>111.2593959569931</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B20" s="4">
+        <v>6924</v>
+      </c>
+      <c r="C20" s="4">
+        <v>346</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5">
+        <v>52.678081726577865</v>
+      </c>
+      <c r="G20" s="5">
+        <v>56.615646326312479</v>
+      </c>
+      <c r="H20" s="5">
+        <v>55.904778723410111</v>
+      </c>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="6">
+        <v>936.37265000000002</v>
+      </c>
+      <c r="N20" s="6">
+        <v>1181.3776499999999</v>
+      </c>
+      <c r="O20" s="6">
+        <v>1755.1333</v>
+      </c>
+      <c r="P20" s="6">
+        <v>2705.3650000000002</v>
+      </c>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" s="4">
+        <v>6924</v>
+      </c>
+      <c r="C21" s="4">
+        <v>415</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5">
+        <v>188.69363637451787</v>
+      </c>
+      <c r="G21" s="5">
+        <v>145.9867377188063</v>
+      </c>
+      <c r="H21" s="5">
+        <v>179.8771638363809</v>
+      </c>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="6">
+        <v>1045.1041</v>
+      </c>
+      <c r="N21" s="6">
+        <v>1249.2117000000001</v>
+      </c>
+      <c r="O21" s="6">
+        <v>1308.6369999999999</v>
+      </c>
+      <c r="P21" s="6">
+        <v>4949.0353000000005</v>
+      </c>
+      <c r="Q21" s="5"/>
+      <c r="R21" s="5"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="4">
+        <v>6738</v>
+      </c>
+      <c r="C22" s="4">
+        <v>226</v>
+      </c>
+      <c r="D22" s="5">
+        <v>8.375837438066398</v>
+      </c>
+      <c r="E22" s="5">
+        <v>1.8258078380468163</v>
+      </c>
+      <c r="F22" s="5">
+        <v>221.91454131031594</v>
+      </c>
+      <c r="G22" s="5">
+        <v>32.085169585070297</v>
+      </c>
+      <c r="H22" s="5">
+        <v>125.40168130104968</v>
+      </c>
+      <c r="I22" s="5">
+        <v>20.408930000000002</v>
+      </c>
+      <c r="J22" s="5">
+        <v>147.76907</v>
+      </c>
+      <c r="K22" s="5">
+        <v>19.878340000000001</v>
+      </c>
+      <c r="L22" s="5">
+        <v>151.95437999999999</v>
+      </c>
+      <c r="M22" s="6">
+        <v>236.35653000000002</v>
+      </c>
+      <c r="N22" s="6">
+        <v>611.37116000000003</v>
+      </c>
+      <c r="O22" s="6">
+        <v>847.86378999999999</v>
+      </c>
+      <c r="P22" s="6">
+        <v>3853.1525199999996</v>
+      </c>
+      <c r="Q22" s="6">
+        <v>8118.7720750570297</v>
+      </c>
+      <c r="R22" s="6">
+        <v>8337.2180815935135</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="4">
+        <v>6738</v>
+      </c>
+      <c r="C23" s="4">
+        <v>249</v>
+      </c>
+      <c r="D23" s="5">
+        <v>4.5591393716669266</v>
+      </c>
+      <c r="E23" s="5">
+        <v>13.937400798256931</v>
+      </c>
+      <c r="F23" s="5">
+        <v>139.41455730235262</v>
+      </c>
+      <c r="G23" s="5">
+        <v>170.22163805974395</v>
+      </c>
+      <c r="H23" s="5">
+        <v>162.85342403036563</v>
+      </c>
+      <c r="I23" s="5">
+        <v>60.446440000000003</v>
+      </c>
+      <c r="J23" s="5">
+        <v>149.67930000000001</v>
+      </c>
+      <c r="K23" s="5">
+        <v>218.04015999999999</v>
+      </c>
+      <c r="L23" s="5">
+        <v>205.01472000000001</v>
+      </c>
+      <c r="M23" s="6">
+        <v>246.89005</v>
+      </c>
+      <c r="N23" s="6">
+        <v>196.01089999999999</v>
+      </c>
+      <c r="O23" s="6">
+        <v>485.25693000000001</v>
+      </c>
+      <c r="P23" s="6">
+        <v>572.85771</v>
+      </c>
+      <c r="Q23" s="6">
+        <v>7013.1572124958038</v>
+      </c>
+      <c r="R23" s="6">
+        <v>9267.8991589546204</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B24" s="4">
+        <v>6738</v>
+      </c>
+      <c r="C24" s="4">
+        <v>320</v>
+      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5">
+        <v>182.92547724741635</v>
+      </c>
+      <c r="G24" s="5">
+        <v>154.56824991140761</v>
+      </c>
+      <c r="H24" s="5">
+        <v>92.575792500002308</v>
+      </c>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="6">
+        <v>560.48519999999996</v>
+      </c>
+      <c r="N24" s="6">
+        <v>563.25936249999995</v>
+      </c>
+      <c r="O24" s="6">
+        <v>833.715735</v>
+      </c>
+      <c r="P24" s="6">
+        <v>2184.3778425</v>
+      </c>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B25" s="4">
+        <v>6740</v>
+      </c>
+      <c r="C25" s="4">
+        <v>226</v>
+      </c>
+      <c r="D25" s="5">
+        <v>5.54740285344712</v>
+      </c>
+      <c r="E25" s="5">
+        <v>4.6901234415333803</v>
+      </c>
+      <c r="F25" s="5">
+        <v>185.87537662166184</v>
+      </c>
+      <c r="G25" s="5">
+        <v>74.892209372931291</v>
+      </c>
+      <c r="H25" s="5">
+        <v>102.18609901412987</v>
+      </c>
+      <c r="I25" s="5">
+        <v>53.24297</v>
+      </c>
+      <c r="J25" s="5">
+        <v>98.859759999999994</v>
+      </c>
+      <c r="K25" s="5">
+        <v>75.760769999999994</v>
+      </c>
+      <c r="L25" s="5">
+        <v>195.67322999999999</v>
+      </c>
+      <c r="M25" s="6">
+        <v>354.68795</v>
+      </c>
+      <c r="N25" s="6">
+        <v>618.56185000000005</v>
+      </c>
+      <c r="O25" s="6">
+        <v>494.27345000000003</v>
+      </c>
+      <c r="P25" s="6">
+        <v>1035.1909499999999</v>
+      </c>
+      <c r="Q25" s="6">
+        <v>573.64939510822296</v>
+      </c>
+      <c r="R25" s="6">
+        <v>395.04139029979706</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A26" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="4">
+        <v>6740</v>
+      </c>
+      <c r="C26" s="4">
+        <v>249</v>
+      </c>
+      <c r="D26" s="5">
+        <v>4.1987913688265612</v>
+      </c>
+      <c r="E26" s="5">
+        <v>2.8741961196456516</v>
+      </c>
+      <c r="F26" s="5">
+        <v>218.43107590101087</v>
+      </c>
+      <c r="G26" s="5">
+        <v>105.86359235238152</v>
+      </c>
+      <c r="H26" s="5">
+        <v>113.77509217671127</v>
+      </c>
+      <c r="I26" s="5">
+        <v>65.873069999999998</v>
+      </c>
+      <c r="J26" s="5">
+        <v>101.64131999999999</v>
+      </c>
+      <c r="K26" s="5">
+        <v>85.894189999999995</v>
+      </c>
+      <c r="L26" s="5">
+        <v>240.58497</v>
+      </c>
+      <c r="M26" s="6">
+        <v>614.12094999999999</v>
+      </c>
+      <c r="N26" s="6">
+        <v>522.07425000000001</v>
+      </c>
+      <c r="O26" s="6">
+        <v>529.58635000000004</v>
+      </c>
+      <c r="P26" s="6">
+        <v>581.74630000000002</v>
+      </c>
+      <c r="Q26" s="6">
+        <v>2273.3482702970505</v>
+      </c>
+      <c r="R26" s="6">
+        <v>1742.9411283731461</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B27" s="4">
+        <v>6740</v>
+      </c>
+      <c r="C27" s="4">
+        <v>320</v>
+      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5">
+        <v>32.59943974626534</v>
+      </c>
+      <c r="G27" s="5">
+        <v>69.098627440874807</v>
+      </c>
+      <c r="H27" s="5">
+        <v>34.944378771198018</v>
+      </c>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="6">
+        <v>471.85982000000001</v>
+      </c>
+      <c r="N27" s="6">
+        <v>1061.8701599999999</v>
+      </c>
+      <c r="O27" s="6">
+        <v>993.74883</v>
+      </c>
+      <c r="P27" s="6">
+        <v>5252.3867200000004</v>
+      </c>
+      <c r="Q27" s="5"/>
+      <c r="R27" s="5"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B28" s="4">
+        <v>6876</v>
+      </c>
+      <c r="C28" s="4">
+        <v>305</v>
+      </c>
+      <c r="D28" s="5">
+        <v>9.896340824030986</v>
+      </c>
+      <c r="E28" s="5">
+        <v>5.9514380275520802</v>
+      </c>
+      <c r="F28" s="5">
+        <v>191.84104477365707</v>
+      </c>
+      <c r="G28" s="5">
+        <v>183.20202316794939</v>
+      </c>
+      <c r="H28" s="5">
+        <v>179.94177131336602</v>
+      </c>
+      <c r="I28" s="5">
+        <v>51.447839999999999</v>
+      </c>
+      <c r="J28" s="5">
+        <v>103.49845999999999</v>
+      </c>
+      <c r="K28" s="5">
+        <v>41.896000000000001</v>
+      </c>
+      <c r="L28" s="5">
+        <v>113.69</v>
+      </c>
+      <c r="M28" s="6">
+        <v>366.65952499999997</v>
+      </c>
+      <c r="N28" s="6">
+        <v>584.51856499999997</v>
+      </c>
+      <c r="O28" s="6">
+        <v>771.96304499999997</v>
+      </c>
+      <c r="P28" s="6">
+        <v>1804.0013300000003</v>
+      </c>
+      <c r="Q28" s="6">
+        <v>223.81388413906097</v>
+      </c>
+      <c r="R28" s="6">
+        <v>87.614457011222839</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="4">
+        <v>6876</v>
+      </c>
+      <c r="C29" s="4">
+        <v>328</v>
+      </c>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5">
+        <v>98.57744087288944</v>
+      </c>
+      <c r="G29" s="5">
+        <v>77.648036327433687</v>
+      </c>
+      <c r="H29" s="5">
+        <v>22.045975075071624</v>
+      </c>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="6"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" s="4">
+        <v>6876</v>
+      </c>
+      <c r="C30" s="4">
+        <v>351</v>
+      </c>
+      <c r="D30" s="5"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5">
+        <v>44.441185361345283</v>
+      </c>
+      <c r="G30" s="5">
+        <v>53.626097096344395</v>
+      </c>
+      <c r="H30" s="5">
+        <v>51.853430656053625</v>
+      </c>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="6"/>
+      <c r="N30" s="6"/>
+      <c r="O30" s="6"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="5"/>
+      <c r="R30" s="5"/>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B31" s="4">
+        <v>6877</v>
+      </c>
+      <c r="C31" s="4">
+        <v>305</v>
+      </c>
+      <c r="D31" s="5">
+        <v>4.9600305117650016</v>
+      </c>
+      <c r="E31" s="5">
+        <v>18.642518939310087</v>
+      </c>
+      <c r="F31" s="5">
+        <v>111.11522831215412</v>
+      </c>
+      <c r="G31" s="5">
+        <v>63.410348482896168</v>
+      </c>
+      <c r="H31" s="5">
+        <v>131.63814108781355</v>
+      </c>
+      <c r="I31" s="5">
+        <v>53.24297</v>
+      </c>
+      <c r="J31" s="5">
+        <v>123.13096</v>
+      </c>
+      <c r="K31" s="5">
+        <v>63.527000000000001</v>
+      </c>
+      <c r="L31" s="5">
+        <v>121.50700000000001</v>
+      </c>
+      <c r="M31" s="6">
+        <v>392.96873499999998</v>
+      </c>
+      <c r="N31" s="6">
+        <v>330.66663499999999</v>
+      </c>
+      <c r="O31" s="6">
+        <v>1935.51647</v>
+      </c>
+      <c r="P31" s="6">
+        <v>2687.8141799999999</v>
+      </c>
+      <c r="Q31" s="6">
+        <v>152.63354110717773</v>
+      </c>
+      <c r="R31" s="6">
+        <v>87.496076226234436</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A32" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B32" s="4">
+        <v>6877</v>
+      </c>
+      <c r="C32" s="4">
+        <v>328</v>
+      </c>
+      <c r="D32" s="5">
+        <v>13.176563169755628</v>
+      </c>
+      <c r="E32" s="5">
+        <v>10.435053471453498</v>
+      </c>
+      <c r="F32" s="5">
+        <v>76.293875505536803</v>
+      </c>
+      <c r="G32" s="5">
+        <v>70.162985834627932</v>
+      </c>
+      <c r="H32" s="5">
+        <v>109.79714564239167</v>
+      </c>
+      <c r="I32" s="5">
+        <v>48.75947</v>
+      </c>
+      <c r="J32" s="5">
+        <v>100.71357999999999</v>
+      </c>
+      <c r="K32" s="5">
+        <v>240.58497</v>
+      </c>
+      <c r="L32" s="5">
+        <v>338.95049999999998</v>
+      </c>
+      <c r="M32" s="6">
+        <v>360.89474999999999</v>
+      </c>
+      <c r="N32" s="6">
+        <v>270.94824999999997</v>
+      </c>
+      <c r="O32" s="6">
+        <v>547.00829999999996</v>
+      </c>
+      <c r="P32" s="6">
+        <v>254.88499999999999</v>
+      </c>
+      <c r="Q32" s="6">
+        <v>7028.7246506214142</v>
+      </c>
+      <c r="R32" s="6">
+        <v>4592.3432430028915</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" s="4">
+        <v>6877</v>
+      </c>
+      <c r="C33" s="4">
+        <v>407</v>
+      </c>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5">
+        <v>59.307088778435329</v>
+      </c>
+      <c r="G33" s="5">
+        <v>24.470737507861891</v>
+      </c>
+      <c r="H33" s="5">
+        <v>136.23733949708705</v>
+      </c>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="6">
+        <v>596.463075</v>
+      </c>
+      <c r="N33" s="6">
+        <v>671.810025</v>
+      </c>
+      <c r="O33" s="6">
+        <v>721.73233500000003</v>
+      </c>
+      <c r="P33" s="6">
+        <v>1477.1434824999999</v>
+      </c>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A34" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B34" s="4">
+        <v>6899</v>
+      </c>
+      <c r="C34" s="4">
+        <v>313</v>
+      </c>
+      <c r="D34" s="5"/>
+      <c r="E34" s="5"/>
+      <c r="F34" s="5">
+        <v>67.168602592974281</v>
+      </c>
+      <c r="G34" s="5">
+        <v>81.842383431106043</v>
+      </c>
+      <c r="H34" s="5">
+        <v>76.920238029181206</v>
+      </c>
+      <c r="I34" s="5">
+        <v>49.65502</v>
+      </c>
+      <c r="J34" s="5">
+        <v>123.13096</v>
+      </c>
+      <c r="K34" s="5">
+        <v>109.00139</v>
+      </c>
+      <c r="L34" s="5">
+        <v>300.09413500000005</v>
+      </c>
+      <c r="M34" s="6">
+        <v>523.32929999999999</v>
+      </c>
+      <c r="N34" s="6">
+        <v>323.52992999999998</v>
+      </c>
+      <c r="O34" s="6">
+        <v>4182.8502600000002</v>
+      </c>
+      <c r="P34" s="6">
+        <v>6396.5856649999996</v>
+      </c>
+      <c r="Q34" s="5"/>
+      <c r="R34" s="5"/>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A35" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" s="4">
+        <v>6899</v>
+      </c>
+      <c r="C35" s="4">
+        <v>336</v>
+      </c>
+      <c r="D35" s="5">
+        <v>1.8225190137226481</v>
+      </c>
+      <c r="E35" s="5">
+        <v>4.2290312535150534</v>
+      </c>
+      <c r="F35" s="5">
+        <v>114.27368888392458</v>
+      </c>
+      <c r="G35" s="5">
+        <v>122.20062508279945</v>
+      </c>
+      <c r="H35" s="5">
+        <v>118.41371348922758</v>
+      </c>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5">
+        <v>68.902699999999996</v>
+      </c>
+      <c r="L35" s="5">
+        <v>246.04883000000001</v>
+      </c>
+      <c r="M35" s="6">
+        <v>208.95095000000001</v>
+      </c>
+      <c r="N35" s="6">
+        <v>201.17805000000001</v>
+      </c>
+      <c r="O35" s="6">
+        <v>307.53095000000002</v>
+      </c>
+      <c r="P35" s="6">
+        <v>290.40445</v>
+      </c>
+      <c r="Q35" s="6">
+        <v>972.15174269676208</v>
+      </c>
+      <c r="R35" s="6">
+        <v>884.70083248615265</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A36" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="4">
+        <v>6899</v>
+      </c>
+      <c r="C36" s="4">
+        <v>407</v>
+      </c>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5">
+        <v>76.439706010930081</v>
+      </c>
+      <c r="G36" s="5">
+        <v>78.590781149796015</v>
+      </c>
+      <c r="H36" s="5">
+        <v>58.18843209150775</v>
+      </c>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+      <c r="L36" s="5"/>
+      <c r="M36" s="6">
+        <v>585.24937499999999</v>
+      </c>
+      <c r="N36" s="6">
+        <v>619.22109999999998</v>
+      </c>
+      <c r="O36" s="6">
+        <v>873.61685499999999</v>
+      </c>
+      <c r="P36" s="6">
+        <v>2104.0159250000002</v>
+      </c>
+      <c r="Q36" s="5"/>
+      <c r="R36" s="5"/>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A37" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" s="4">
+        <v>6903</v>
+      </c>
+      <c r="C37" s="4">
+        <v>313</v>
+      </c>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5">
+        <v>73.233254652903099</v>
+      </c>
+      <c r="G37" s="5">
+        <v>40.877662699055584</v>
+      </c>
+      <c r="H37" s="5">
+        <v>50.525383850864081</v>
+      </c>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5">
+        <v>46.358870000000003</v>
+      </c>
+      <c r="L37" s="5">
+        <v>141.7878</v>
+      </c>
+      <c r="M37" s="6">
+        <v>432.90530000000001</v>
+      </c>
+      <c r="N37" s="6">
+        <v>553.06686000000002</v>
+      </c>
+      <c r="O37" s="6">
+        <v>1546.1052299999999</v>
+      </c>
+      <c r="P37" s="6">
+        <v>4949.2402899999997</v>
+      </c>
+      <c r="Q37" s="5"/>
+      <c r="R37" s="5"/>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A38" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" s="4">
+        <v>6943</v>
+      </c>
+      <c r="C38" s="4">
+        <v>328</v>
+      </c>
+      <c r="D38" s="5">
+        <v>10.657700849319133</v>
+      </c>
+      <c r="E38" s="5">
+        <v>2.4578538684726956</v>
+      </c>
+      <c r="F38" s="5">
+        <v>132.25918963782081</v>
+      </c>
+      <c r="G38" s="5">
+        <v>95.259524387760862</v>
+      </c>
+      <c r="H38" s="5">
+        <v>129.67553324594223</v>
+      </c>
+      <c r="I38" s="5">
+        <v>85.026949999999999</v>
+      </c>
+      <c r="J38" s="5">
+        <v>145.86098000000001</v>
+      </c>
+      <c r="K38" s="5">
+        <v>65.991500000000002</v>
+      </c>
+      <c r="L38" s="5">
+        <v>310.04056000000003</v>
+      </c>
+      <c r="M38" s="6">
+        <v>685.93105000000003</v>
+      </c>
+      <c r="N38" s="6">
+        <v>614.43685000000005</v>
+      </c>
+      <c r="O38" s="6">
+        <v>2531.1384950000001</v>
+      </c>
+      <c r="P38" s="6">
+        <v>4151.4012199999997</v>
+      </c>
+      <c r="Q38" s="6">
+        <v>8874.9001741409302</v>
+      </c>
+      <c r="R38" s="6">
+        <v>8322.3337959051132</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A39" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39" s="4">
+        <v>6943</v>
+      </c>
+      <c r="C39" s="4">
+        <v>351</v>
+      </c>
+      <c r="D39" s="5"/>
+      <c r="E39" s="5"/>
+      <c r="F39" s="5">
+        <v>31.320643119115328</v>
+      </c>
+      <c r="G39" s="5">
+        <v>53.994216576244234</v>
+      </c>
+      <c r="H39" s="5">
+        <v>81.238010439079588</v>
+      </c>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+      <c r="L39" s="5"/>
+      <c r="M39" s="6">
+        <v>605.95475499999998</v>
+      </c>
+      <c r="N39" s="6">
+        <v>690.52542000000005</v>
+      </c>
+      <c r="O39" s="6">
+        <v>2387.1781774999999</v>
+      </c>
+      <c r="P39" s="6">
+        <v>3168.7369250000002</v>
+      </c>
+      <c r="Q39" s="5"/>
+      <c r="R39" s="5"/>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A40" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B40" s="4">
+        <v>6943</v>
+      </c>
+      <c r="C40" s="4">
+        <v>422</v>
+      </c>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5">
+        <v>129.49460939318027</v>
+      </c>
+      <c r="G40" s="5">
+        <v>122.79047128086302</v>
+      </c>
+      <c r="H40" s="5">
+        <v>154.63426315489679</v>
+      </c>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+      <c r="L40" s="5"/>
+      <c r="M40" s="6">
+        <v>1116.635</v>
+      </c>
+      <c r="N40" s="6">
+        <v>1239.8838000000001</v>
+      </c>
+      <c r="O40" s="6">
+        <v>977.40300000000002</v>
+      </c>
+      <c r="P40" s="6">
+        <v>775.1454</v>
+      </c>
+      <c r="Q40" s="5"/>
+      <c r="R40" s="5"/>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A41" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B41" s="4">
+        <v>6949</v>
+      </c>
+      <c r="C41" s="4">
+        <v>328</v>
+      </c>
+      <c r="D41" s="5">
+        <v>0.72013639883430025</v>
+      </c>
+      <c r="E41" s="5">
+        <v>11.396842997345848</v>
+      </c>
+      <c r="F41" s="5">
+        <v>113.82166967795088</v>
+      </c>
+      <c r="G41" s="5">
+        <v>77.226589110002891</v>
+      </c>
+      <c r="H41" s="5">
+        <v>81.176974332151772</v>
+      </c>
+      <c r="I41" s="5">
+        <v>50.551139999999997</v>
+      </c>
+      <c r="J41" s="5">
+        <v>142.05117999999999</v>
+      </c>
+      <c r="K41" s="5">
+        <v>165.04948999999999</v>
+      </c>
+      <c r="L41" s="5">
+        <v>254.41738000000001</v>
+      </c>
+      <c r="M41" s="6">
+        <v>225.11525</v>
+      </c>
+      <c r="N41" s="6">
+        <v>191.88114999999999</v>
+      </c>
+      <c r="O41" s="6">
+        <v>343.6345</v>
+      </c>
+      <c r="P41" s="6">
+        <v>270.14370000000002</v>
+      </c>
+      <c r="Q41" s="6">
+        <v>7982.0121800899506</v>
+      </c>
+      <c r="R41" s="6">
+        <v>8774.7569861412048</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="I42" s="4"/>
+      <c r="J42" s="4"/>
+      <c r="M42" s="6"/>
+      <c r="N42" s="6"/>
+      <c r="O42" s="6"/>
+      <c r="P42" s="6"/>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869A4FAA-CE51-4079-B8C9-E1049BD3D220}">
   <dimension ref="A1:X41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="28.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -6861,12 +8855,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1381C3B9-FC7C-48B1-8B93-856E9C87ACD7}">
   <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.5703125" customWidth="1"/>
+    <col min="2" max="2" width="49.7109375" customWidth="1"/>
     <col min="3" max="3" width="18.85546875" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>